<commit_message>
Only one screw length
</commit_message>
<xml_diff>
--- a/accessories/cable-1/cable-1.xlsx
+++ b/accessories/cable-1/cable-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c0fa0fe96562a9e/Documents/GitHub/Battery-Lab-Hardware/accessories/cable-1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{00529C85-C1FB-4B8D-8F8E-701A9C9B067D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B08AE21-A859-440D-9224-0CB17283EA62}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{00529C85-C1FB-4B8D-8F8E-701A9C9B067D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{238A80B5-4592-4200-97EC-E835F6C3AEC0}"/>
   <bookViews>
-    <workbookView xWindow="30615" yWindow="1815" windowWidth="21600" windowHeight="11055" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11055" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="68">
   <si>
     <t>Individual Cost</t>
   </si>
@@ -239,19 +239,7 @@
     <t>https://www.grainger.com/product/Hex-Nut-Std-Hex-26KR85?searchQuery=M01300.030.0001&amp;searchBar=true&amp;tier=Tier+6&amp;suggestConfigId=6&amp;s_e=false</t>
   </si>
   <si>
-    <t>SBS75 Handle Screws Short</t>
-  </si>
-  <si>
-    <t>Standard Socket Head Cap Screw: M3x0.50, 18 mm Lg, Std, Black Oxide, Alloy Steel, Class 12.9, 100 PK</t>
-  </si>
-  <si>
-    <t>M07000.030.0018</t>
-  </si>
-  <si>
-    <t>https://www.grainger.com/product/Standard-Socket-Head-Cap-Screw-6CE54</t>
-  </si>
-  <si>
-    <t>SBS75 Handle Screws Long</t>
+    <t>SBS75 Handle Screws</t>
   </si>
 </sst>
 </file>
@@ -940,7 +928,7 @@
         <v>2.4</v>
       </c>
       <c r="F7" s="9">
-        <f t="shared" ref="F7:F13" si="1">D7*E7</f>
+        <f t="shared" ref="F7:F12" si="1">D7*E7</f>
         <v>4.8</v>
       </c>
       <c r="G7" s="5"/>
@@ -1106,7 +1094,7 @@
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>60</v>
@@ -1115,13 +1103,13 @@
         <v>61</v>
       </c>
       <c r="D14" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="8">
         <v>0.37</v>
       </c>
       <c r="F14" s="9">
-        <v>0.37</v>
+        <v>0.94</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="3" t="s">
@@ -1131,54 +1119,40 @@
       <c r="J14" s="11"/>
     </row>
     <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>67</v>
+      <c r="A15" s="16" t="s">
+        <v>63</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D15" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="13">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
       <c r="F15" s="9">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
       <c r="G15" s="11"/>
       <c r="H15" s="17" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="I15" s="11"/>
       <c r="J15" s="11"/>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="D16" s="12">
-        <v>2</v>
-      </c>
-      <c r="E16" s="13">
-        <v>0.04</v>
-      </c>
-      <c r="F16" s="9">
-        <v>0.08</v>
-      </c>
+      <c r="A16" s="16"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="9"/>
       <c r="G16" s="11"/>
-      <c r="H16" s="17" t="s">
-        <v>66</v>
-      </c>
+      <c r="H16" s="17"/>
     </row>
     <row r="17" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E17" s="8"/>
@@ -1190,7 +1164,7 @@
       </c>
       <c r="F18" s="5">
         <f>SUM(F2:F17)</f>
-        <v>258.42000000000007</v>
+        <v>258.88000000000005</v>
       </c>
     </row>
   </sheetData>
@@ -1209,7 +1183,7 @@
     <hyperlink ref="H10" r:id="rId11" xr:uid="{1563652D-3B5B-4137-B0DA-8740E4BAA28B}"/>
     <hyperlink ref="H11" r:id="rId12" xr:uid="{8810426D-4117-48F2-9859-A19CAA6ADB2C}"/>
     <hyperlink ref="H12" r:id="rId13" xr:uid="{CCA64CC5-DC08-4003-9DCA-627D9167BE5E}"/>
-    <hyperlink ref="H16" r:id="rId14" xr:uid="{DBEFA464-01ED-4E2E-BC80-A2D024432206}"/>
+    <hyperlink ref="H15" r:id="rId14" xr:uid="{2CA896D6-A65A-4B3D-8048-6D965D3E69AC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId15"/>

</xml_diff>